<commit_message>
Updated calculations and added COCOMO I & II Calculations for Sprint 4
</commit_message>
<xml_diff>
--- a/Evidence/PP/COCOMO I and II Calculations/COCOMO I & II Calculations Sprint 4.xlsx
+++ b/Evidence/PP/COCOMO I and II Calculations/COCOMO I & II Calculations Sprint 4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neelp\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF5C1B41-E6B7-4138-BF2D-EE5090A37E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9397977-381F-4EFE-9510-F5A198030B14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28965" yWindow="-165" windowWidth="29130" windowHeight="16530" xr2:uid="{8C05499B-E777-4CB1-ACAA-0667EC699DC3}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="10240" xr2:uid="{8C05499B-E777-4CB1-ACAA-0667EC699DC3}"/>
   </bookViews>
   <sheets>
     <sheet name="COCOMO I and II" sheetId="1" r:id="rId1"/>
@@ -239,16 +239,16 @@
     <t>Values</t>
   </si>
   <si>
-    <t>player time</t>
-  </si>
-  <si>
-    <t>player config</t>
-  </si>
-  <si>
-    <t>user data</t>
-  </si>
-  <si>
-    <t>player io</t>
+    <t>player_time.py</t>
+  </si>
+  <si>
+    <t>player_config.py</t>
+  </si>
+  <si>
+    <t>user_data.py</t>
+  </si>
+  <si>
+    <t>player_io.py</t>
   </si>
 </sst>
 </file>

</xml_diff>